<commit_message>
Apply FY27 budget assumptions
</commit_message>
<xml_diff>
--- a/templates/00_Template_Index.xlsx
+++ b/templates/00_Template_Index.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Index" sheetId="1" r:id="Rd8b3bb8c3aab47c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Index" sheetId="1" r:id="R07a13a04b9834a27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -239,7 +239,7 @@
         <x:v>Venue count</x:v>
       </x:c>
       <x:c r="B3" t="n">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>